<commit_message>
auto: atualiza base operacional via atalho
</commit_message>
<xml_diff>
--- a/data/status_saida/operacional/status_set_2026.xlsx
+++ b/data/status_saida/operacional/status_set_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\opera\Desktop\app\dashboard_operacao\data\status_saida\operacional\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{475EE138-26E0-4B5A-B7DE-E2F02DED5560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{35F3D634-E624-48A6-9CA7-C491F4BCBA0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D2AC9CA4-D229-4570-A7F7-D6EE9B8F4085}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FDE459A8-8443-404D-84A7-2A7BF2285522}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -18763,7 +18763,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4862ED67-94FC-459E-8EE1-DCBB6E631695}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7B3E211-C069-46F6-A726-AB22990CF98B}">
   <dimension ref="A1:Y724"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>

</xml_diff>